<commit_message>
Upload clean project files from Day 5 to Day 10
</commit_message>
<xml_diff>
--- a/Month-1/Day-5/Naanaa_Sales_Dashboard.xlsx
+++ b/Month-1/Day-5/Naanaa_Sales_Dashboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data-Analysis-and-AI-85Days\Month-1\Day-5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BED30DD9-09CC-4130-AB5A-F9636EC8125C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E07962C-05EE-4D59-9234-0E22A17A9CB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{088B5373-8884-4FE4-ABB3-E5C60BDE4D4F}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId2"/>
+    <pivotCache cacheId="27" r:id="rId2"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -2036,10 +2036,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="ahmed" refreshedDate="46203.896709259257" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="10" xr:uid="{5E1E4272-A09D-47B3-800F-63CE7423B8D0}">
   <cacheSource type="worksheet">
@@ -2164,7 +2160,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{24B44A4E-E266-4761-9183-85972786ACFF}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{24B44A4E-E266-4761-9183-85972786ACFF}" name="PivotTable1" cacheId="27" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
   <location ref="H4:I10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="5">
     <pivotField showAll="0"/>
@@ -2979,9 +2975,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3129,26 +3128,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F25F156-FAE9-47FD-9EB4-FA484B3E124E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DD48C94-0A90-475F-BC5F-2A791FA2F63C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="d6bf451c-e3aa-4dd1-b5a6-a95183d31bdf"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3172,9 +3160,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7DD48C94-0A90-475F-BC5F-2A791FA2F63C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5F25F156-FAE9-47FD-9EB4-FA484B3E124E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="d6bf451c-e3aa-4dd1-b5a6-a95183d31bdf"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>